<commit_message>
Sync project updates 2026-10-13 14:03:32 +01:00
</commit_message>
<xml_diff>
--- a/02_检索与核验记录/特殊科研资助清单_20261013/机器人相关特殊科研资助清单_20261013.xlsx
+++ b/02_检索与核验记录/特殊科研资助清单_20261013/机器人相关特殊科研资助清单_20261013.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\桌面\全国机器人与医工开放项目\02_检索与核验记录\特殊科研资助清单_20261013\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DCA591C-1F45-46C7-8674-9D4DE32E9CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E50460-6F06-4969-A4A3-F86B8795459B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
   <si>
     <t>机器人相关科研资助与合作渠道</t>
   </si>
@@ -28,18 +28,12 @@
     <t>截至2026-10-13；7项保留渠道、3项待定。截止按北京时间；未知字段留空，具体缺口见最后一列。</t>
   </si>
   <si>
-    <t>核验状态</t>
-  </si>
-  <si>
     <t>项目／具体方向</t>
   </si>
   <si>
     <t>截止日期（北京时间）</t>
   </si>
   <si>
-    <t>受理时间说明</t>
-  </si>
-  <si>
     <t>经费及资金口径</t>
   </si>
   <si>
@@ -58,27 +52,6 @@
     <t>尚缺资料</t>
   </si>
   <si>
-    <t>任务相关</t>
-  </si>
-  <si>
-    <t>智能算力与先进测控专项·A06</t>
-  </si>
-  <si>
-    <t>一般课题研究经费5—25万元；软硬件平台支持另计。</t>
-  </si>
-  <si>
-    <t>智能制造与具身机器人智能测控；包含机器人感知控制、视觉测控、实时算力调度及测控系统，须体现算力应用。</t>
-  </si>
-  <si>
-    <t>面向全国高校；团队不少于3人；每位申报人限报1项；有可使用的基础软硬件，外部资源须说明；学校签章，成果知识产权共有。</t>
-  </si>
-  <si>
-    <t>申请书自行约定成果、技术指标、提交方式与时间，按约定完成；已读附件未规定统一论文、专利或样机数量。</t>
-  </si>
-  <si>
-    <t>团队、具体题目与实验资源尚未由本人确认。</t>
-  </si>
-  <si>
     <t>西安第四批创新挑战·需求163</t>
   </si>
   <si>
@@ -97,15 +70,9 @@
     <t>具体截止时刻未载；当前需求承接状态、合同、分工及经费尚待落实。</t>
   </si>
   <si>
-    <t>任务相关（口腔场景）</t>
-  </si>
-  <si>
     <t>北京联合基金·海淀医学人工智能培育6</t>
   </si>
   <si>
-    <t>16:00</t>
-  </si>
-  <si>
     <t>30万元／项目，3年。</t>
   </si>
   <si>
@@ -121,15 +88,9 @@
     <t>北京依托关系、年度申请及团队限项、医学场景资源尚待本人确认。</t>
   </si>
   <si>
-    <t>任务相关（规划／视觉反馈）</t>
-  </si>
-  <si>
     <t>郑州企业出题·高新领域第1项</t>
   </si>
   <si>
-    <t>18:00；推荐截至11月29日18:00</t>
-  </si>
-  <si>
     <t>企业总投入／企业出资100万元，2年；高校合同经费另议。财政后补对象为企业，≤已支付攻关额50%。</t>
   </si>
   <si>
@@ -145,9 +106,6 @@
     <t>技术合同、投入时间、成果权属与落地安排尚待落实。</t>
   </si>
   <si>
-    <t>任务相关（定位／软件）</t>
-  </si>
-  <si>
     <t>体育科技需求·第31项</t>
   </si>
   <si>
@@ -164,54 +122,6 @@
   </si>
   <si>
     <t>具体截止时刻未载；需求单位、合同额、具体控制任务与指标尚待对接。</t>
-  </si>
-  <si>
-    <t>自主选题渠道</t>
-  </si>
-  <si>
-    <t>国自然原创探索计划·专家推荐类</t>
-  </si>
-  <si>
-    <t>全年受理</t>
-  </si>
-  <si>
-    <t>预算按方案提出；既有指南一般1—3年、≤100万元／年；非固定拨款额度。</t>
-  </si>
-  <si>
-    <t>可自主提出机器人控制基础研究；须具有原创探索、非共识及高风险特征。</t>
-  </si>
-  <si>
-    <t>需2名符合指南要求的推荐人；全年限申请1项，含预申请；核心内容不得与在研或评审中项目重复。普通控制课题不能仅换名称申报。</t>
-  </si>
-  <si>
-    <t>按批准的研究方案、任务与项目管理要求执行。</t>
-  </si>
-  <si>
-    <t>推荐人、年度申请及原创探索方案尚未确认；具体结题条款需按获准项目进一步核对。</t>
-  </si>
-  <si>
-    <t>自主选题合作渠道</t>
-  </si>
-  <si>
-    <t>江西2027自然基金·20万元重点类别</t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>20万元，3—4年；合作经费安排另核。</t>
-  </si>
-  <si>
-    <t>自主基础研究，可由当地团队提出机器人控制与建模科学问题；非已指定的机器人任务。</t>
-  </si>
-  <si>
-    <t>主持人≤58岁，须有国自然主持经历，满足学历／职称等要求；须江西固定人员牵头，本人以南信大合作参与。不得兼职或挂靠主持；当地负责人及参与者限项另核。</t>
-  </si>
-  <si>
-    <t>当地负责人、合作安排、限项、经费分配及具体结题条件尚未落实／核清。</t>
-  </si>
-  <si>
-    <t>待定</t>
   </si>
   <si>
     <t>泸州2026科技计划</t>
@@ -255,7 +165,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -291,14 +201,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF24446A"/>
-      <name val="Microsoft YaHei"/>
-      <family val="2"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
@@ -323,7 +225,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -342,22 +244,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFE9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFF3F6FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7EDF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -372,10 +259,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -388,25 +275,16 @@
     <xf numFmtId="176" fontId="3" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -429,12 +307,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingChannels" displayName="FundingChannels" ref="A5:J15" totalsRowShown="0">
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="核验状态"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingChannels" displayName="FundingChannels" ref="A5:H12" totalsRowShown="0">
+  <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="项目／具体方向"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="截止日期（北京时间）"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="受理时间说明"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="经费及资金口径"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="实际研究方向"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="申请条件及待落实事项"/>
@@ -644,7 +520,7 @@
   <sheetPr>
     <tabColor rgb="FF24446A"/>
   </sheetPr>
-  <dimension ref="A2:J15"/>
+  <dimension ref="A2:J12"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -712,306 +588,175 @@
       <c r="H5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="6" spans="1:10" ht="105" customHeight="1">
       <c r="A6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="7">
+        <v>46325</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="E6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="5">
-        <v>46402</v>
-      </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="4" t="s">
+    </row>
+    <row r="7" spans="1:10" ht="105" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="B7" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J6" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" ht="105" customHeight="1">
-      <c r="A7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="7" t="s">
+      <c r="E7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="8">
-        <v>46325</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="G7" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="105" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="7">
+        <v>46353</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="F8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="5">
-        <v>46321</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="G8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="4" t="s">
+    </row>
+    <row r="9" spans="1:10" ht="105" customHeight="1">
+      <c r="A9" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="B9" s="5">
+        <v>46326</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="I8" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J8" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="105" customHeight="1">
-      <c r="A9" s="6" t="s">
+      <c r="G9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="7" t="s">
+    </row>
+    <row r="10" spans="1:10" ht="94.95" customHeight="1">
+      <c r="A10" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="8">
-        <v>46353</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="7" t="s">
+    </row>
+    <row r="11" spans="1:10" ht="94.95" customHeight="1">
+      <c r="A11" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="B11" s="5"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="F11" s="4"/>
+      <c r="G11" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="7" t="s">
+    </row>
+    <row r="12" spans="1:10" ht="94.95" customHeight="1">
+      <c r="A12" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="J9" s="7" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="105" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="5">
-        <v>46326</v>
-      </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="105" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="105" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="5">
-        <v>46324</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H12" s="4"/>
-      <c r="I12" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="94.95" customHeight="1">
-      <c r="A13" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="94.95" customHeight="1">
-      <c r="A14" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="H14" s="4"/>
-      <c r="I14" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="94.95" customHeight="1">
-      <c r="A15" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="C15" s="8"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="I6" r:id="rId1" display="https://www.cutech.edu.cn/detail/46-838" xr:uid="{846E29B2-7CE7-44D3-A17D-2860C0631EED}"/>
-    <hyperlink ref="I7" r:id="rId2" display="https://xakj.xa.gov.cn/kjdt/tzgg/2105191117492449281.html" xr:uid="{A7BC6D2D-481B-443C-A4B8-99EA0829605B}"/>
-    <hyperlink ref="I8" r:id="rId3" display="https://kw.beijing.gov.cn/zwgk/zcwj/202609/t20260929_4885502.html" xr:uid="{DEAEAA50-1F87-4D46-8D9F-14AFED6D68C3}"/>
-    <hyperlink ref="I9" r:id="rId4" display="https://zzkj.zhengzhou.gov.cn/tzgg/10251173.jhtml" xr:uid="{C1E70CE9-A3B7-4950-B045-666A0A3C48A1}"/>
-    <hyperlink ref="I10" r:id="rId5" display="https://www.sport.gov.cn/n315/n20001395/c30068905/content.html" xr:uid="{11B6450D-B3E3-4572-930B-0E262F9CD69F}"/>
-    <hyperlink ref="I11" r:id="rId6" display="https://www.nsfc.gov.cn/p1/3381/2824/101332.html" xr:uid="{96DFB9EE-2D14-40A6-B063-DA2444730ED5}"/>
-    <hyperlink ref="I12" r:id="rId7" display="https://kyc.jxufe.edu.cn/news-show-9071.html" xr:uid="{87F1678C-1CFA-4910-BEA0-B989121F5B11}"/>
-    <hyperlink ref="I13" r:id="rId8" display="https://kjc.swmu.edu.cn/info/1032/11772.htm" xr:uid="{11C94229-05D7-4EC8-8CE9-5F2F606C7E24}"/>
-    <hyperlink ref="I14" r:id="rId9" display="https://qdstc.qingdao.gov.cn/kjdt/tzgg/202609/t20260929_10744647.shtml" xr:uid="{11A8C1E7-1522-4DB5-898A-38F08F27CE35}"/>
-    <hyperlink ref="I15" r:id="rId10" display="https://bulletin.nuist.edu.cn/content.jsp?urltype=news.NewsContentUrl&amp;wbnewsid=57793&amp;wbtreeid=1015" xr:uid="{6D58F3A7-B7E5-4093-931A-B659DEF79155}"/>
+    <hyperlink ref="G6" r:id="rId1" display="https://xakj.xa.gov.cn/kjdt/tzgg/2105191117492449281.html" xr:uid="{A7BC6D2D-481B-443C-A4B8-99EA0829605B}"/>
+    <hyperlink ref="G7" r:id="rId2" display="https://kw.beijing.gov.cn/zwgk/zcwj/202609/t20260929_4885502.html" xr:uid="{DEAEAA50-1F87-4D46-8D9F-14AFED6D68C3}"/>
+    <hyperlink ref="G8" r:id="rId3" display="https://zzkj.zhengzhou.gov.cn/tzgg/10251173.jhtml" xr:uid="{C1E70CE9-A3B7-4950-B045-666A0A3C48A1}"/>
+    <hyperlink ref="G9" r:id="rId4" display="https://www.sport.gov.cn/n315/n20001395/c30068905/content.html" xr:uid="{11B6450D-B3E3-4572-930B-0E262F9CD69F}"/>
+    <hyperlink ref="G10" r:id="rId5" display="https://kjc.swmu.edu.cn/info/1032/11772.htm" xr:uid="{11C94229-05D7-4EC8-8CE9-5F2F606C7E24}"/>
+    <hyperlink ref="G11" r:id="rId6" display="https://qdstc.qingdao.gov.cn/kjdt/tzgg/202609/t20260929_10744647.shtml" xr:uid="{11A8C1E7-1522-4DB5-898A-38F08F27CE35}"/>
+    <hyperlink ref="G12" r:id="rId7" display="https://bulletin.nuist.edu.cn/content.jsp?urltype=news.NewsContentUrl&amp;wbnewsid=57793&amp;wbtreeid=1015" xr:uid="{6D58F3A7-B7E5-4093-931A-B659DEF79155}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync project updates 2026-10-13 14:25:28 +01:00
</commit_message>
<xml_diff>
--- a/02_检索与核验记录/特殊科研资助清单_20261013/机器人相关特殊科研资助清单_20261013.xlsx
+++ b/02_检索与核验记录/特殊科研资助清单_20261013/机器人相关特殊科研资助清单_20261013.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\桌面\全国机器人与医工开放项目\02_检索与核验记录\特殊科研资助清单_20261013\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66E50460-6F06-4969-A4A3-F86B8795459B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E634F6-30EB-48E2-9235-227D2A2BD3A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,14 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
   <si>
     <t>机器人相关科研资助与合作渠道</t>
   </si>
   <si>
-    <t>截至2026-10-13；7项保留渠道、3项待定。截止按北京时间；未知字段留空，具体缺口见最后一列。</t>
-  </si>
-  <si>
     <t>项目／具体方向</t>
   </si>
   <si>
@@ -122,27 +119,6 @@
   </si>
   <si>
     <t>具体截止时刻未载；需求单位、合同额、具体控制任务与指标尚待对接。</t>
-  </si>
-  <si>
-    <t>泸州2026科技计划</t>
-  </si>
-  <si>
-    <t>附件1完整指南未取得；全市截止、机器人任务、金额、资格及结题条件未核清。10月26日是西南医大校内截止，未填作本项目截止。</t>
-  </si>
-  <si>
-    <t>青岛2027科技惠民／关键技术攻关</t>
-  </si>
-  <si>
-    <t>关键技术攻关由企业牵头，高校可合作参与；科技惠民与攻关类别具体要求分别核。</t>
-  </si>
-  <si>
-    <t>平台权限受限，具体方向指南未取得；机器人任务、对应类别截止、经费及结题条件待核。已取得学校通知中的10月22日17:00窗口明确针对科技惠民，尚未逐类别核到，未填为两类共同截止。</t>
-  </si>
-  <si>
-    <t>江苏科技副总（南信大通知）</t>
-  </si>
-  <si>
-    <t>校内通知及企业岗位／技术需求目录未取得；截止、具体机器人任务、研究经费、申请及考核条件待核。</t>
   </si>
   <si>
     <r>
@@ -307,7 +283,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingChannels" displayName="FundingChannels" ref="A5:H12" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FundingChannels" displayName="FundingChannels" ref="A5:H10" totalsRowShown="0">
   <tableColumns count="8">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="项目／具体方向"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="截止日期（北京时间）"/>
@@ -520,7 +496,7 @@
   <sheetPr>
     <tabColor rgb="FF24446A"/>
   </sheetPr>
-  <dimension ref="A2:J12"/>
+  <dimension ref="A2:J10"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -550,9 +526,7 @@
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" ht="24" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -565,183 +539,143 @@
     </row>
     <row r="5" spans="1:10" ht="36" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="105" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="7">
         <v>46325</v>
       </c>
       <c r="C6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="105" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" s="5">
         <v>46321</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="105" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="7">
         <v>46353</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="G8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="105" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="5">
         <v>46326</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="10" spans="1:10" ht="94.95" customHeight="1">
-      <c r="A10" s="6" t="s">
-        <v>34</v>
-      </c>
+      <c r="A10" s="6"/>
       <c r="B10" s="7"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
-      <c r="G10" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="94.95" customHeight="1">
-      <c r="A11" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="94.95" customHeight="1">
-      <c r="A12" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="G10" s="9"/>
+      <c r="H10" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -750,13 +684,10 @@
     <hyperlink ref="G7" r:id="rId2" display="https://kw.beijing.gov.cn/zwgk/zcwj/202609/t20260929_4885502.html" xr:uid="{DEAEAA50-1F87-4D46-8D9F-14AFED6D68C3}"/>
     <hyperlink ref="G8" r:id="rId3" display="https://zzkj.zhengzhou.gov.cn/tzgg/10251173.jhtml" xr:uid="{C1E70CE9-A3B7-4950-B045-666A0A3C48A1}"/>
     <hyperlink ref="G9" r:id="rId4" display="https://www.sport.gov.cn/n315/n20001395/c30068905/content.html" xr:uid="{11B6450D-B3E3-4572-930B-0E262F9CD69F}"/>
-    <hyperlink ref="G10" r:id="rId5" display="https://kjc.swmu.edu.cn/info/1032/11772.htm" xr:uid="{11C94229-05D7-4EC8-8CE9-5F2F606C7E24}"/>
-    <hyperlink ref="G11" r:id="rId6" display="https://qdstc.qingdao.gov.cn/kjdt/tzgg/202609/t20260929_10744647.shtml" xr:uid="{11A8C1E7-1522-4DB5-898A-38F08F27CE35}"/>
-    <hyperlink ref="G12" r:id="rId7" display="https://bulletin.nuist.edu.cn/content.jsp?urltype=news.NewsContentUrl&amp;wbnewsid=57793&amp;wbtreeid=1015" xr:uid="{6D58F3A7-B7E5-4093-931A-B659DEF79155}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>